<commit_message>
Casos PMD1: nombres realistas en Excel 01-15 y bases SQLite/CSV 01-16 (mismos IDs, cifras y errores intencionales) + script renombrar_nombres_reales.py
</commit_message>
<xml_diff>
--- a/PMD1_15_Casos_Sinteticos/09_Clinica_PMD1.xlsx
+++ b/PMD1_15_Casos_Sinteticos/09_Clinica_PMD1.xlsx
@@ -18812,7 +18812,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Cliente 1</t>
+          <t>Víctor Paredes Castillo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -18832,7 +18832,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cliente 2</t>
+          <t>Diana Mamani Cárdenas</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -18852,7 +18852,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Cliente 3</t>
+          <t>Óscar Campos Gómez</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -18872,7 +18872,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cliente 4</t>
+          <t>Ana Mendoza Salazar</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -18892,7 +18892,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Cliente 5</t>
+          <t>Luis Salazar Ríos</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -18912,7 +18912,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Cliente 6</t>
+          <t>María Valdivia Rojas</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -18932,7 +18932,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Cliente 7</t>
+          <t>Jorge Cruz Espinoza</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -18952,7 +18952,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Cliente 8</t>
+          <t>Rosa Huamán Cruz</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -18972,7 +18972,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cliente 9</t>
+          <t>Carlos Ramírez Castillo</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -18992,7 +18992,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cliente 10</t>
+          <t>Lucía Aguilar Cárdenas</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -19012,7 +19012,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cliente 11</t>
+          <t>Miguel Navarro Gómez</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -19032,7 +19032,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cliente 12</t>
+          <t>Carmen Quispe Ramírez</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -19052,7 +19052,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Cliente 13</t>
+          <t>José Torres Condori</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -19072,7 +19072,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cliente 14</t>
+          <t>Patricia Espinoza Flores</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -19092,7 +19092,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Cliente 15</t>
+          <t>Diego Poma Paredes</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -19112,7 +19112,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cliente 16</t>
+          <t>Milagros Gómez Navarro</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -19132,7 +19132,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Cliente 17</t>
+          <t>Renzo Vargas Mendoza</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -19152,7 +19152,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Cliente 18</t>
+          <t>Gabriela Paredes Delgado</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -19172,7 +19172,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cliente 19  </t>
+          <t xml:space="preserve">Hugo Mamani Campos  </t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -19192,7 +19192,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Cliente 20</t>
+          <t>Fiorella Campos Torres</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -19212,7 +19212,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Cliente 21</t>
+          <t>César Rojas Valdivia</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -19232,7 +19232,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cliente 22</t>
+          <t>Paola Gutiérrez Benites</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -19252,7 +19252,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Cliente 23</t>
+          <t>Iván Cárdenas Gutiérrez</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -19272,7 +19272,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Cliente 24</t>
+          <t>Sofía Soto Poma</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -19292,7 +19292,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Cliente 25</t>
+          <t>Martín Flores Huamán</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -19312,7 +19312,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Cliente 26</t>
+          <t>Elena Chávez Ccori</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -19332,7 +19332,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Cliente 27</t>
+          <t>Raúl Delgado Soto</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -19352,7 +19352,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Cliente 28</t>
+          <t>Valeria Ríos Vargas</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -19372,7 +19372,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Cliente 29</t>
+          <t>Andrés Benites Aguilar</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -19392,7 +19392,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Cliente 30</t>
+          <t>Claudia Castillo Reyes</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -19412,7 +19412,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Cliente 31</t>
+          <t>Víctor Ccori Chávez</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -19432,7 +19432,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Cliente 32</t>
+          <t>Diana Condori Mamani</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -19452,7 +19452,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Cliente 33</t>
+          <t>Óscar Reyes Quispe</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -19472,7 +19472,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Cliente 34</t>
+          <t>Ana Vargas Ccori</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -19492,7 +19492,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Cliente 35</t>
+          <t>Luis Paredes Soto</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -19512,7 +19512,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Cliente 36</t>
+          <t>María Mamani Vargas</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -19532,7 +19532,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cliente 37</t>
+          <t>Jorge Campos Aguilar</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -19552,7 +19552,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cliente 38  </t>
+          <t xml:space="preserve">Rosa Rojas Reyes  </t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -19572,7 +19572,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cliente 39</t>
+          <t>Carlos Gutiérrez Chávez</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -19592,7 +19592,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Cliente 40</t>
+          <t>Lucía Cárdenas Mamani</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -19612,7 +19612,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Cliente 41</t>
+          <t>Miguel Soto Quispe</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -19632,7 +19632,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Cliente 42</t>
+          <t>Carmen Flores Salazar</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -19652,7 +19652,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Cliente 43</t>
+          <t>José Chávez Ríos</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -19672,7 +19672,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Cliente 44</t>
+          <t>Patricia Delgado Rojas</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -19692,7 +19692,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Cliente 45</t>
+          <t>Diego Ríos Espinoza</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -19712,7 +19712,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Cliente 46</t>
+          <t>Milagros Benites Cruz</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -19732,7 +19732,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Cliente 47</t>
+          <t>Gabriela Ccori Cárdenas</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -19752,7 +19752,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Cliente 48</t>
+          <t>Hugo Condori Gómez</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -19772,7 +19772,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Cliente 49</t>
+          <t>Fiorella Reyes Ramírez</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -19792,7 +19792,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Cliente 50</t>
+          <t>César Mendoza Condori</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -19812,7 +19812,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Cliente 51</t>
+          <t>Paola Salazar Flores</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -19832,7 +19832,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Cliente 52</t>
+          <t>Iván Valdivia Paredes</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -19852,7 +19852,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Cliente 53</t>
+          <t>Sofía Cruz Navarro</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -19872,7 +19872,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Cliente 54</t>
+          <t>Martín Huamán Mendoza</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -19892,7 +19892,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Cliente 55</t>
+          <t>Elena Ramírez Delgado</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -19912,7 +19912,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cliente 56</t>
+          <t>Raúl Aguilar Campos</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -19932,7 +19932,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cliente 57  </t>
+          <t xml:space="preserve">Valeria Navarro Torres  </t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -19952,7 +19952,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Cliente 58</t>
+          <t>Andrés Quispe Valdivia</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -19972,7 +19972,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Cliente 59</t>
+          <t>Claudia Torres Benites</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -19992,7 +19992,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Cliente 60</t>
+          <t>Víctor Espinoza Gutiérrez</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -20012,7 +20012,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Cliente 61</t>
+          <t>Óscar Gómez Huamán</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -20032,7 +20032,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Cliente 62</t>
+          <t>Ana Castillo Delgado</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -20052,7 +20052,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Cliente 63</t>
+          <t>Luis Ccori Campos</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -20072,7 +20072,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Cliente 64</t>
+          <t>María Condori Torres</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -20092,7 +20092,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Cliente 65</t>
+          <t>Jorge Reyes Valdivia</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -20112,7 +20112,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Cliente 66</t>
+          <t>Rosa Mendoza Benites</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -20132,7 +20132,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Cliente 67</t>
+          <t>Carlos Salazar Gutiérrez</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -20152,7 +20152,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Cliente 68</t>
+          <t>Lucía Valdivia Poma</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -20172,7 +20172,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Cliente 69</t>
+          <t>Miguel Cruz Huamán</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -20192,7 +20192,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Cliente 70</t>
+          <t>Carmen Huamán Ccori</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -20212,7 +20212,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Cliente 71</t>
+          <t>José Ramírez Soto</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -20232,7 +20232,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Cliente 72</t>
+          <t>Patricia Aguilar Vargas</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -20252,7 +20252,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Cliente 73</t>
+          <t>Diego Navarro Aguilar</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -20272,7 +20272,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Cliente 74</t>
+          <t>Milagros Quispe Reyes</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -20292,7 +20292,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Cliente 75</t>
+          <t>Renzo Torres Chávez</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -20312,7 +20312,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cliente 76  </t>
+          <t xml:space="preserve">Gabriela Espinoza Mamani  </t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -20332,7 +20332,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Cliente 77</t>
+          <t>Hugo Poma Quispe</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -20352,7 +20352,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Cliente 78</t>
+          <t>Fiorella Gómez Salazar</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -20372,7 +20372,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Cliente 79</t>
+          <t>César Vargas Ríos</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -20392,7 +20392,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Cliente 80</t>
+          <t>Paola Paredes Rojas</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -20412,7 +20412,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Cliente 81</t>
+          <t>Iván Mamani Espinoza</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -20432,7 +20432,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Cliente 82</t>
+          <t>Sofía Campos Cruz</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -20452,7 +20452,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Cliente 83</t>
+          <t>Martín Rojas Castillo</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -20472,7 +20472,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Cliente 84</t>
+          <t>Elena Gutiérrez Cárdenas</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -20492,7 +20492,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Cliente 85</t>
+          <t>Raúl Cárdenas Gómez</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -20512,7 +20512,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Cliente 86</t>
+          <t>Valeria Soto Ramírez</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -20532,7 +20532,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Cliente 87</t>
+          <t>Andrés Flores Condori</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -20552,7 +20552,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Cliente 88</t>
+          <t>Claudia Chávez Flores</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -20572,7 +20572,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Cliente 89</t>
+          <t>Víctor Delgado Paredes</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -20592,7 +20592,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Cliente 90</t>
+          <t>Diana Ríos Navarro</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -20612,7 +20612,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Cliente 91</t>
+          <t>Óscar Benites Mendoza</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -20632,7 +20632,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Cliente 92</t>
+          <t>Ana Torres Cárdenas</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -20652,7 +20652,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Cliente 93</t>
+          <t>Luis Espinoza Gómez</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -20672,7 +20672,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Cliente 94</t>
+          <t>María Poma Ramírez</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -20692,7 +20692,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cliente 95  </t>
+          <t xml:space="preserve">Jorge Gómez Condori  </t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -20712,7 +20712,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Cliente 96</t>
+          <t>Rosa Vargas Flores</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -20732,7 +20732,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Cliente 97</t>
+          <t>Lucía Mamani Navarro</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -20752,7 +20752,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Cliente 98</t>
+          <t>Miguel Campos Mendoza</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -20772,7 +20772,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Cliente 99</t>
+          <t>Carmen Rojas Delgado</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -20792,7 +20792,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Cliente 100</t>
+          <t>José Gutiérrez Campos</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -20812,7 +20812,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Cliente 101</t>
+          <t>Patricia Cárdenas Torres</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -20832,7 +20832,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Cliente 102</t>
+          <t>Diego Soto Valdivia</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -20852,7 +20852,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Cliente 103</t>
+          <t>Milagros Flores Benites</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -20872,7 +20872,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Cliente 104</t>
+          <t>Renzo Chávez Gutiérrez</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -20892,7 +20892,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Cliente 105</t>
+          <t>Gabriela Delgado Poma</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -20912,7 +20912,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Cliente 106</t>
+          <t>Hugo Ríos Huamán</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -20932,7 +20932,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Cliente 107</t>
+          <t>Fiorella Benites Ccori</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -20952,7 +20952,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Cliente 108</t>
+          <t>César Castillo Soto</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -20972,7 +20972,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Cliente 109</t>
+          <t>Paola Ccori Vargas</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -20992,7 +20992,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Cliente 110</t>
+          <t>Iván Condori Aguilar</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -21012,7 +21012,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Cliente 111</t>
+          <t>Martín Mendoza Chávez</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -21032,7 +21032,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Cliente 112</t>
+          <t>Elena Salazar Mamani</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -21052,7 +21052,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Cliente 113</t>
+          <t>Raúl Valdivia Quispe</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -21072,7 +21072,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cliente 114  </t>
+          <t xml:space="preserve">Valeria Cruz Salazar  </t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -21092,7 +21092,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Cliente 115</t>
+          <t>Andrés Huamán Ríos</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -21112,7 +21112,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Cliente 116</t>
+          <t>Claudia Ramírez Rojas</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -21132,7 +21132,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Cliente 117</t>
+          <t>Víctor Aguilar Espinoza</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -21152,7 +21152,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Cliente 118</t>
+          <t>Diana Navarro Cruz</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -21172,7 +21172,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Cliente 119</t>
+          <t>Óscar Quispe Castillo</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -21192,7 +21192,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Cliente 120</t>
+          <t>Ana Chávez Mamani</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -21254,7 +21254,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>control 1</t>
+          <t>Control prenatal</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21274,7 +21274,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>imagen 2</t>
+          <t>Radiografía de tórax</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -21294,7 +21294,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>terapia 3</t>
+          <t>Terapia física</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -21314,7 +21314,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>analisis 4</t>
+          <t>Hemograma completo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -21334,7 +21334,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>imagen 5</t>
+          <t>Ecografía abdominal</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -21354,7 +21354,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>consulta 6</t>
+          <t>Consulta de medicina general</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -21374,7 +21374,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>control 7</t>
+          <t>Control de niño sano</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -21394,7 +21394,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>terapia 8</t>
+          <t>Terapia de lenguaje</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -21414,7 +21414,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>analisis 9</t>
+          <t>Perfil lipídico</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -21434,7 +21434,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>consulta 10</t>
+          <t>Consulta pediátrica</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -21454,7 +21454,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>imagen 11</t>
+          <t>Tomografía</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -21474,7 +21474,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>analisis 12</t>
+          <t>Glucosa en ayunas</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -21494,7 +21494,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>terapia 13</t>
+          <t>Terapia respiratoria</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -21514,7 +21514,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>control 14</t>
+          <t>Control de presión arterial</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -21534,7 +21534,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>consulta 15</t>
+          <t>Consulta ginecológica</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -21554,7 +21554,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>control 16</t>
+          <t>Control de diabetes</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -21574,7 +21574,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>consulta 17</t>
+          <t>Consulta cardiológica</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -21594,7 +21594,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>terapia 18</t>
+          <t>Rehabilitación de rodilla</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -21614,7 +21614,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>terapia 19</t>
+          <t>Terapia ocupacional</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -21634,7 +21634,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>terapia 20</t>
+          <t>Electroterapia</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -21690,7 +21690,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Clinica sede 1</t>
+          <t>Clínica San Gabriel Los Olivos</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -21707,7 +21707,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Clinica sede 2</t>
+          <t>Clínica San Gabriel San Miguel</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -21724,7 +21724,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Clinica sede 3</t>
+          <t>Clínica San Gabriel La Molina</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -21741,7 +21741,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Clinica sede 4</t>
+          <t>Clínica San Gabriel Callao</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -21758,7 +21758,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Clinica sede 5</t>
+          <t>Clínica San Gabriel Magdalena del Mar</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">

</xml_diff>